<commit_message>
Portfolio Analyser v1.0 - Phase 12 complete
- Full G1/G2/G3 integrated workflow
- 5-scorecard scoring pipeline (Fundamental, Valuation, Technical, Sentiment, Risk)
- ATR-based stop-loss with breach detection
- G2 three-mode discovery (Gap Fill, Peer Compare, Diversifier)
- G3 sector drift detection and rebalancing plan
- Streamlit dashboard with Portfolio Overview and Stock Detail tabs
- Claude AI sentiment layer with source badges
- Excel portfolio import with loop guard
- SQLite cache + portfolio DB
- YAML-driven config with no hardcoded thresholds
</commit_message>
<xml_diff>
--- a/data/input/portfolio.xlsx
+++ b/data/input/portfolio.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nikhilkirtikar/Documents/Nikhil/portfolio_analyser/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A770A5-3F97-A449-9CE6-612DCE2679BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0DDFDC9-61AB-C740-86AD-4CBCB26D6C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2320" yWindow="660" windowWidth="29920" windowHeight="17600" xr2:uid="{CA5E7731-8723-4A42-B0D8-BE355D325723}"/>
+    <workbookView xWindow="0" yWindow="580" windowWidth="34560" windowHeight="17600" xr2:uid="{CA5E7731-8723-4A42-B0D8-BE355D325723}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="53">
   <si>
     <t>Company Name</t>
   </si>
@@ -44,6 +44,72 @@
     <t>Sector</t>
   </si>
   <si>
+    <t>Adani Ports</t>
+  </si>
+  <si>
+    <t>Bombay Burmah</t>
+  </si>
+  <si>
+    <t>FMCG</t>
+  </si>
+  <si>
+    <t>Himadri Special</t>
+  </si>
+  <si>
+    <t>Chemicals</t>
+  </si>
+  <si>
+    <t>Sun Pharma.Inds.</t>
+  </si>
+  <si>
+    <t>Pidilite Inds.</t>
+  </si>
+  <si>
+    <t>Radico Khaitan</t>
+  </si>
+  <si>
+    <t>ADANIPOWER</t>
+  </si>
+  <si>
+    <t>Havells India</t>
+  </si>
+  <si>
+    <t>Titan Company</t>
+  </si>
+  <si>
+    <t>MAZDOCK</t>
+  </si>
+  <si>
+    <t>Bharat Forge</t>
+  </si>
+  <si>
+    <t>HDFC Bank</t>
+  </si>
+  <si>
+    <t>Uno Minda</t>
+  </si>
+  <si>
+    <t>Lumax Auto Tech.</t>
+  </si>
+  <si>
+    <t>Maruti Suzuki</t>
+  </si>
+  <si>
+    <t>J K Cements</t>
+  </si>
+  <si>
+    <t>Vedanta</t>
+  </si>
+  <si>
+    <t>Gabriel India</t>
+  </si>
+  <si>
+    <t>Reliance Industr</t>
+  </si>
+  <si>
+    <t>Tata Consumer</t>
+  </si>
+  <si>
     <t>Ticker</t>
   </si>
   <si>
@@ -53,22 +119,82 @@
     <t>Quantity</t>
   </si>
   <si>
+    <t>ADANIPORTS</t>
+  </si>
+  <si>
+    <t>BBTC</t>
+  </si>
+  <si>
+    <t>HSCL</t>
+  </si>
+  <si>
+    <t>SUNPHARMA</t>
+  </si>
+  <si>
+    <t>PIDILITIND</t>
+  </si>
+  <si>
+    <t>RADICO</t>
+  </si>
+  <si>
+    <t>HAVELLS</t>
+  </si>
+  <si>
+    <t>TITAN</t>
+  </si>
+  <si>
+    <t>BHARATFORG</t>
+  </si>
+  <si>
+    <t>HDFCBANK</t>
+  </si>
+  <si>
+    <t>UNOMINDA</t>
+  </si>
+  <si>
+    <t>LUMAXTECH</t>
+  </si>
+  <si>
+    <t>MARUTI</t>
+  </si>
+  <si>
+    <t>JKCEMENT</t>
+  </si>
+  <si>
+    <t>VEDL</t>
+  </si>
+  <si>
+    <t>GABRIEL</t>
+  </si>
+  <si>
+    <t>RELIANCE</t>
+  </si>
+  <si>
+    <t>TATACONSUM</t>
+  </si>
+  <si>
     <t>Infrastructure</t>
   </si>
   <si>
+    <t>Energy</t>
+  </si>
+  <si>
     <t>Automobile</t>
   </si>
   <si>
-    <t>J K Cements</t>
-  </si>
-  <si>
-    <t>Lumax Auto Tech.</t>
-  </si>
-  <si>
-    <t>JKCEMENT</t>
-  </si>
-  <si>
-    <t>LUMAXTECH</t>
+    <t>Consumer</t>
+  </si>
+  <si>
+    <t>Financial Services</t>
+  </si>
+  <si>
+    <t>Shipbullding</t>
+  </si>
+  <si>
+    <t>Pharma</t>
+  </si>
+  <si>
+    <t>SHRIRAMFIN</t>
   </si>
 </sst>
 </file>
@@ -111,7 +237,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -119,16 +245,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -465,65 +610,389 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7E7BB60-675F-1A4E-9C20-6F68E7134638}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="17.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="12.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="4">
+        <v>1597.5</v>
+      </c>
+      <c r="E2" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="4">
+        <v>194.41</v>
+      </c>
+      <c r="E3" s="2">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="4">
+        <v>1477.53</v>
+      </c>
+      <c r="E4" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="D5" s="4">
+        <v>1555.77</v>
+      </c>
+      <c r="E5" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="4">
+        <v>472.72</v>
+      </c>
+      <c r="E6" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1299.3</v>
+      </c>
+      <c r="E7" s="2">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="4">
+        <v>467.96</v>
+      </c>
+      <c r="E8" s="2">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="4">
+        <v>526.65</v>
+      </c>
+      <c r="E9" s="2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2983.14</v>
+      </c>
+      <c r="E10" s="2">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1687.47</v>
+      </c>
+      <c r="E11" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D12" s="4">
+        <v>12282.66</v>
+      </c>
+      <c r="E12" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2066.73</v>
+      </c>
+      <c r="E13" s="2">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="4">
+        <v>737.48</v>
+      </c>
+      <c r="E14" s="2">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C15" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2328.42</v>
+      </c>
+      <c r="E15" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="4">
+        <v>602.02</v>
+      </c>
+      <c r="E16" s="2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1021.17</v>
+      </c>
+      <c r="E17" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="2">
-        <v>2983.14</v>
-      </c>
-      <c r="E2" s="2">
+      <c r="C18" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" s="4">
+        <v>1673.33</v>
+      </c>
+      <c r="E18" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1132.68</v>
+      </c>
+      <c r="E19" s="2">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="4">
+        <v>2739.22</v>
+      </c>
+      <c r="E20" s="2">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1687.47</v>
-      </c>
-      <c r="E3" s="2">
-        <v>5</v>
+      <c r="C21" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="4">
+        <v>463.04</v>
+      </c>
+      <c r="E21" s="2">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" s="4">
+        <v>702.98</v>
+      </c>
+      <c r="E22" s="2">
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>